<commit_message>
actualizacion de las correcciones en correspondencia con los datos del anexo 1 y la tesis de referencia
</commit_message>
<xml_diff>
--- a/output/catalogo_variables.xlsx
+++ b/output/catalogo_variables.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Datos" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -429,35 +429,50 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Descripcion_funcional</t>
+          <t>Unidad</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Unidad</t>
+          <t>Tipo_dato</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Tipo_dato</t>
+          <t>Tipo_en_modelo</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>Mecanismos_asociados</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Ecuacion</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Rol_en_ecuacion</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
           <t>Rango_min</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Rango_max</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Distribucion_observada</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Pregunta_planta</t>
         </is>
@@ -476,33 +491,48 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Nivel de exigencia operativa del sistema, influyendo directamente en los esfuerzos aplicados y en la probabilidad de fallo</t>
+          <t>MW</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>MW</t>
+          <t>float</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
+          <t>Carga</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Vibraciones_mecanicas,HCF (High Cycle Fatigue)</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>G(X) = C - D (estado limite, Nachlas 1995)</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Potencia de salida que induce esfuerzos mecanicos sobre el rotor. Participa en funcion de estado limite G(X) = Capacidad - Demanda. Referencia: Perez (2024), Nachlas (1995)</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
         <v>263.56</v>
       </c>
-      <c r="G2" t="n">
+      <c r="J2" t="n">
         <v>272.11</v>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Distribución multimodal, aproximadamente simétrica, colas cortas (platicúrtica), baja dispersión</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Frecuencia de muestreo?, Descripcion?</t>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Weibull (forma=132.4, escala=269.6), asimetrica positiva, colas largas, KS p-value=0.71</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>¿Ubicacion del sensor? ¿Medicion directa o calculada? ¿Frecuencia de muestreo? ¿Precision? ¿Ultima calibracion? ¿Retrasos?</t>
         </is>
       </c>
     </row>
@@ -514,38 +544,53 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>flujo_vapor_sobrecalentado_cuerpo_ap_turbina</t>
+          <t>flujo_vapor_sobrecalentado</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Caudal de vapor que incide en la turbina, determinando los esfuerzos térmicos y mecánicos sobre sus componentes</t>
+          <t>t/h</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>t/h</t>
+          <t>float</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
+          <t>Carga</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>SPE (Solid Particle Erosion)</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>sigma_y = 1.14e-7 * rho_ox * d_ox^3 * (F_v/S)^2 - Ecs (2.1),(2.11),(2.15),(2.16),(2.17)</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>F_v en energia cinetica para erosion SPE. rho_ox=5.08 g/cm³, d_ox via oxidacion parabolica. Constantes: A=6.22e20 µm²/h, Eox=-326kJ/mol. Referencia: Perez (2024), Reshetnyak (1995)</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
         <v>774.38</v>
       </c>
-      <c r="G3" t="n">
+      <c r="J3" t="n">
         <v>788.41</v>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Distribución multimodal, asimétrica negativa (cola izquierda), colas largas (leptocúrtica), baja dispersión</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Frecuencia de muestreo?, Descripcion?</t>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Weibull (forma=321.4, escala=785.4), asimetrica positiva, colas largas, KS p-value=0.98</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>¿Ubicacion? ¿Directa o calculada? ¿Frecuencia? ¿Precision? ¿Calibracion? ¿Retrasos de transporte?</t>
         </is>
       </c>
     </row>
@@ -557,38 +602,53 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>temp_vapor_sobrecalentado_despues_atemperador_izq</t>
+          <t>temp_vapor_sobrecalentado_atemperador</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Nivel térmico del vapor, determinando los esfuerzos térmicos y el riesgo de degradación de los componentes</t>
+          <t>°C</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>°C</t>
+          <t>float</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
+          <t>Carga</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Choque_termico,Fatiga_termica</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Nu = 0.023 * Re^0.8 * Pr^n (Dittus-Boelter) - Ecs (2.25),(2.27),(2.28)</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>T entrada para coeficiente de pelicula y numero de Nusselt. n=0.4 calentamiento, n=0.02 calentamiento real. Referencia: Perez (2024), Leyzerovich (2008)</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
         <v>401.19</v>
       </c>
-      <c r="G4" t="n">
+      <c r="J4" t="n">
         <v>403.35</v>
       </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Distribución multimodal, aproximadamente simétrica, colas cortas (platicúrtica), baja dispersión</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Frecuencia de muestreo?, Descripcion?</t>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Weibull (forma=685.8, escala=402.6), asimetrica positiva, colas cortas, KS p-value=0.34</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>¿Ubicacion? ¿Contacto directo? ¿Frecuencia? ¿Precision? ¿Calibracion? ¿Retraso termico?</t>
         </is>
       </c>
     </row>
@@ -600,38 +660,53 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>temp_vapor_recalentado_salida_caldera</t>
+          <t>temp_vapor_recalentado_salida</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Nivel térmico del vapor recalentado, influyendo en los esfuerzos térmicos y en la probabilidad de fallo de los componentes</t>
+          <t>°C</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>°C</t>
+          <t>float</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="F5" t="n">
+          <t>Carga</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Creep (Fluencia lenta),Fatiga_termica</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>LMP = T*(C + log10(t_r)) - Ecs (2.8),(2.9),(2.12),(2.32)</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>T absoluta para parametro Larson-Miller, C=20, en vida remanente por creep. Influye en oxidacion parabolica. Referencia: Perez (2024), Mendelson (1965)</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
         <v>535.14</v>
       </c>
-      <c r="G5" t="n">
+      <c r="J5" t="n">
         <v>538.88</v>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Distribución multimodal, aproximadamente simétrica, colas cortas (platicúrtica), baja dispersión</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>Frecuencia de muestreo?, Descripcion?</t>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Weibull (forma=479.2, escala=537.6), asimetrica positiva, colas cortas, KS p-value=0.48</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>¿Ubicacion? ¿Directa? ¿Frecuencia? ¿Precision? ¿Calibracion? ¿Influencia de radiacion?</t>
         </is>
       </c>
     </row>
@@ -643,38 +718,53 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>pres_domo</t>
+          <t>presion_domo</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Nivel de presión del sistema, influyendo en los esfuerzos mecánicos y en la probabilidad de fallo de los componentes</t>
+          <t>bar</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>bar</t>
+          <t>float</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="F6" t="n">
+          <t>Carga</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Creep,SCC (Stress Corrosion Cracking)</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>sigma_theta = P*r/t (esfuerzo circunferencial)</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>P genera esfuerzos de membrana en paredes del domo para analisis de creep y SCC. sigma_theta = P*r/t. Referencia: Perez (2024)</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
         <v>171.45</v>
       </c>
-      <c r="G6" t="n">
+      <c r="J6" t="n">
         <v>174.16</v>
       </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Distribución multimodal, asimétrica negativa (cola izquierda), colas largas (leptocúrtica), baja dispersión</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Frecuencia de muestreo?, Descripcion?</t>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Normal (mu=173.2, sigma=0.62), simetrica, colas cortas, KS p-value=0.94</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>¿Ubicacion? ¿Directa? ¿Frecuencia? ¿Precision? ¿Calibracion? ¿Pulsaciones?</t>
         </is>
       </c>
     </row>
@@ -686,38 +776,53 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>pres_vap_sobrecal_a_turbina</t>
+          <t>presion_vapor_sobrecalentado_turbina</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Presión del vapor de entrada, determinando los esfuerzos mecánicos y el riesgo de fallo en los componentes</t>
+          <t>bar</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>bar</t>
+          <t>float</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="F7" t="n">
-        <v>165.28</v>
-      </c>
-      <c r="G7" t="n">
+          <t>Carga</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>SPE,Creep</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>V = F_v/S, rho_corregida = f(P,T) - Ecs (2.14),(2.19)</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>P_tr entrada para correccion de densidad del vapor y calculo de velocidad V = F_v/S. Influye en energia cinetica de SPE. Referencia: Perez (2024)</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>164.26</v>
+      </c>
+      <c r="J7" t="n">
         <v>166.8</v>
       </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>Distribución multimodal, asimétrica negativa (cola izquierda), colas largas (leptocúrtica), baja dispersión</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>Frecuencia de muestreo?, Descripcion?</t>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Gamma (forma=78396, escala=0.002), asimetrica positiva, colas cortas, KS p-value=0.96</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>¿Ubicacion? ¿Directa? ¿Frecuencia? ¿Precision? ¿Calibracion? ¿Vibraciones?</t>
         </is>
       </c>
     </row>
@@ -729,38 +834,459 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>pres_vapor_entrada_recalentador</t>
+          <t>presion_vapor_entrada_recalentador</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Presión del vapor antes del recalentamiento, influyendo en los esfuerzos mecánicos y en la probabilidad de fallo de los componentes</t>
+          <t>bar</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>bar</t>
+          <t>float</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="F8" t="n">
+          <t>Carga</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Creep,Oxidacion</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>d_ox^2 = 2*A*exp(-Eox/(R*T))*dt - Ecs (2.10),(2.36),(2.37),(2.38)</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>P_T entrada para calculo de espesor de oxido d_ox via oxidacion parabolica. Constantes: A=6.22e20 µm²/h, Eox=-326kJ/mol. Influye en sigma_y para SPE. Referencia: Sabau (2014), Perez (2024)</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
         <v>29.51</v>
       </c>
-      <c r="G8" t="n">
+      <c r="J8" t="n">
         <v>30.38</v>
       </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Distribución multimodal, aproximadamente simétrica, colas cortas (platicúrtica), baja dispersión</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>Frecuencia de muestreo?, Descripcion?</t>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Gamma (forma=10723, escala=0.003), asimetrica positiva, colas cortas, KS p-value=0.71</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>¿Ubicacion? ¿Directa? ¿Frecuencia? ¿Precision? ¿Calibracion? ¿Humedad?</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Acero_1CrMoV_LimFluencia</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>limite_fluencia_acero_rotor</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>MPa</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Resistencia</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>SPE,Creep,Fatiga_termica,SCC</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>sigma_y_resistencia = sigma_y (Perez 2024)</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>sigma_y=240 MPa resistencia superficial contra erosion SPE. Composicion segun ASTM A470. Tratamiento: Austenizacion 850-900C, Revenido 540-680C. Referencia: Perez (2024), ASM Handbook</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>240</v>
+      </c>
+      <c r="J9" t="n">
+        <v>240</v>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Composicion: C=0.28-0.35%, Cr=0.90-1.20%, Mo=0.20-0.35%, V=0.05-0.15%. Trat: Austeniz 850-900C + Revenido 540-680C. Certificados: ASTM A470, ASME Section II. Ubicacion probetas: zona rotor, eje</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Acero_1CrMoV_ResFatiga</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>resistencia_fatiga_acero</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>MPa</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Resistencia</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Fatiga_termica,Vibraciones_mecanicas</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>sigma_n = Ca*Cb*Cc*Cd*Ce*sigma_n_prim (Anexo 6)</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Resistencia a fatiga corregida. Coeficientes: Ca=0.75 (superficial), Cb=0.85 (tamano eje 550mm), Cc=0.82 (confianza 99%), Cd=0.42 (T=540C), Ce=0.99 (entalla). sigma_n_prim=835 MPa teorica. Curva S-N: sigma = 1315 - 0.563*N. Referencia: Anexo 6 tesis, ASM Fatigue Handbook</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>190</v>
+      </c>
+      <c r="J10" t="n">
+        <v>190</v>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Coeficientes: Ca=0.75, Cb=0.85, Cc=0.82, Cd=0.42, Ce=0.99. Curva S-N: sigma=1315-0.563N. Temp. operacion: 530C (800K). Zona probetas: rotor, eje. Norma: ASTM E466</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Acero_1CrMoV_ModElasticidad</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>modulo_elasticidad_acero</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>GPa</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Resistencia</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Vibraciones_mecanicas,Fatiga_termica</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>sigma = E*epsilon (Ley elastica de Hooke)</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Modulo de Young E=160 GPa para calculo de deformaciones elasticas. Degrada &gt;450C. Referencia: Perez (2024), ASM Handbook</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>160</v>
+      </c>
+      <c r="J11" t="n">
+        <v>160</v>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>E=160 GPa a temp. ambiente. Curva E vs T: degradacion &gt;450C. Ensayo a temp. elevada necesario. Tipo: 1CrMoV. Precision: segun ASTM A470</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Acero_1CrMoV_DilTermica</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>coef_dilatacion_termica</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>1/°C</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Resistencia</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Choque_termico,Fatiga_termica</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>delta_L = alpha * L0 * delta_T</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Coeficiente alpha=1.2e-5 1/°C para calculo de deformaciones termicas. Referencia: Pagina 103 tesis</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>1.2e-05</v>
+      </c>
+      <c r="J12" t="n">
+        <v>1.2e-05</v>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Alpha=1.2e-5 1/°C. Ensayo a temp. elevada requerido (&gt;450C). Tipo: 1CrMoV. Precision: segun ASTM A470</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Acero_1CrMoV_Densidad</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>densidad_acero</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>g/cm³</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Resistencia</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>SPE,Vibraciones_mecanicas</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>masa = densidad * volumen</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Densidad=7.8 g/cm³ para calculo de masa y esfuerzos inerciales. Referencia: Pagina 103 tesis</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="J13" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Densidad=7.8 g/cm³ segun ASM Handbook. Ensayo: metodo hidrostatico. Muestra: representativa del rotor. Homogeneidad verificada por certificados ASTM A470</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Acero_1CrMoV_Cp</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>capacidad_calorifica</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>J/kg°C</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Resistencia</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Choque_termico,Fatiga_termica,Creep</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Q = Cp * masa * delta_T</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Capacidad calorifica Cp=680 J/kg°C para transferencia de calor. Degrada &gt;500C. Referencia: Pagina 103 tesis</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>680</v>
+      </c>
+      <c r="J14" t="n">
+        <v>680</v>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>Cp=680 J/kg°C a temp. ambiente. Curva Cp vs T: degradacion &gt;500C. Ensayo: calorimeria diferencial. Norma: ASTM E1269</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Oxido_Fe3O4_Densidad</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>densidad_oxido_magnetita</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>g/cm³</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Resistencia</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>SPE</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>sigma_y = 1.14e-7 * rho_ox * d_ox^3 * (F_v/S)^2</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Densidad oxidos rho_ox=5.08 g/cm³ para erosion SPE. Transforma a hematites &gt;600C. Referencia: Sabau (2014), Dooley (2019)</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>5.08</v>
+      </c>
+      <c r="J15" t="n">
+        <v>5.08</v>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>¿Composicion exacta? ¿Oxidacion? ¿Espesor escama?</t>
         </is>
       </c>
     </row>

</xml_diff>